<commit_message>
feat(decay): parametrize γ decay function + empirical comparison
- Add src/funcs/decay.py with 4 decay variants:
  exponential (default), polynomial, logarithmic, adaptive
- Parametrize GeometricSIA to accept decay_fn=None (fully retrocompatible)
- Add experiments/comparativa_decay.py with benchmark harness
  · Patches SafeLogger and ProfilingManager to avoid I/O overhead
  · Runs 13 cases × 4 variants → results/comparativa_decay.xlsx
- Result: all 52 runs converge to identical MIP — decay influences
  cost table but not final candidate selection on current test cases

Refs: GeoMIP Cap. 6 — 'Factores de decrecimiento alternativos'
</commit_message>
<xml_diff>
--- a/GeoMIP/results/resultados_Geometric.xlsx
+++ b/GeoMIP/results/resultados_Geometric.xlsx
@@ -475,7 +475,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>9,645855188369751</t>
+          <t>9,130457401275635</t>
         </is>
       </c>
     </row>
@@ -506,7 +506,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>8,994643211364746</t>
+          <t>9,947686433792114</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4,819844484329224</t>
+          <t>4,413058519363403</t>
         </is>
       </c>
     </row>
@@ -568,7 +568,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>4,430887937545776</t>
+          <t>5,6272125244140625</t>
         </is>
       </c>
     </row>
@@ -599,7 +599,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>0,1475987434387207</t>
+          <t>0,12518715858459473</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0,10084795951843262</t>
+          <t>0,10082411766052246</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>0,29232311248779297</t>
+          <t>0,300506591796875</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>9,453017234802246</t>
+          <t>9,870303392410278</t>
         </is>
       </c>
     </row>
@@ -723,7 +723,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10,670487880706787</t>
+          <t>9,80565619468689</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>5,1378419399261475</t>
+          <t>4,572464227676392</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>4,1559789180755615</t>
+          <t>3,4125711917877197</t>
         </is>
       </c>
     </row>
@@ -816,7 +816,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0,11781454086303711</t>
+          <t>0,12459993362426758</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0,09478235244750977</t>
+          <t>0,054877281188964844</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0,2680954933166504</t>
+          <t>0,17388153076171875</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>9,850761890411377</t>
+          <t>5,465152978897095</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>10,709792375564575</t>
+          <t>5,441627025604248</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>4,348508596420288</t>
+          <t>2,860286235809326</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>4,476068496704102</t>
+          <t>2,6066219806671143</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0,10819506645202637</t>
+          <t>0,07834720611572266</t>
         </is>
       </c>
     </row>
@@ -1064,7 +1064,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>0,09859323501586914</t>
+          <t>0,05383753776550293</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>0,5535805225372314</t>
+          <t>0,15437054634094238</t>
         </is>
       </c>
     </row>
@@ -1126,7 +1126,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>11,755699634552002</t>
+          <t>5,373405933380127</t>
         </is>
       </c>
     </row>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>9,574047327041626</t>
+          <t>6,309786319732666</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>4,9787187576293945</t>
+          <t>2,7556209564208984</t>
         </is>
       </c>
     </row>
@@ -1219,7 +1219,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>4,829437255859375</t>
+          <t>2,805262565612793</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0,11637330055236816</t>
+          <t>0,08409810066223145</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0,16582655906677246</t>
+          <t>0,04185128211975098</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0,23525643348693848</t>
+          <t>0,12991118431091309</t>
         </is>
       </c>
     </row>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>7,350882053375244</t>
+          <t>3,9679598808288574</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>7,035381078720093</t>
+          <t>3,9771029949188232</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1405,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>3,4193601608276367</t>
+          <t>1,873161792755127</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>3,4474689960479736</t>
+          <t>1,892859697341919</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>0,11075210571289062</t>
+          <t>0,03680229187011719</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>0,08561015129089355</t>
+          <t>0,023342609405517578</t>
         </is>
       </c>
     </row>
@@ -1529,7 +1529,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>0,19605231285095215</t>
+          <t>0,09239411354064941</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>8,690616846084595</t>
+          <t>3,5053188800811768</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>7,590581655502319</t>
+          <t>3,453232526779175</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>3,192997694015503</t>
+          <t>1,5822594165802002</t>
         </is>
       </c>
     </row>
@@ -1653,7 +1653,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>3,142817497253418</t>
+          <t>1,6607844829559326</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>0,06869935989379883</t>
+          <t>0,026947736740112305</t>
         </is>
       </c>
     </row>
@@ -1715,7 +1715,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>0,03729057312011719</t>
+          <t>0,02012038230895996</t>
         </is>
       </c>
     </row>
@@ -1746,7 +1746,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0,16179847717285156</t>
+          <t>0,08850264549255371</t>
         </is>
       </c>
     </row>
@@ -1777,7 +1777,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>7,698806285858154</t>
+          <t>3,8804280757904053</t>
         </is>
       </c>
     </row>
@@ -1808,7 +1808,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>7,6919825077056885</t>
+          <t>3,974909543991089</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1839,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>3,666226863861084</t>
+          <t>1,8571836948394775</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>3,5166568756103516</t>
+          <t>1,8523590564727783</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>0,07656478881835938</t>
+          <t>0,03794717788696289</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>0,061514854431152344</t>
+          <t>0,024960994720458984</t>
         </is>
       </c>
     </row>
@@ -1963,7 +1963,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>0,20150136947631836</t>
+          <t>0,10233139991760254</t>
         </is>
       </c>
     </row>
@@ -1994,7 +1994,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>4,073901414871216</t>
+          <t>2,127455234527588</t>
         </is>
       </c>
     </row>

</xml_diff>